<commit_message>
Parenthesized unions (chart series, SUM((A,B))) expand like argument lists
Found in nested-groups: a chart over two sample group rows turned into #REF!.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/templates/grouped-footers/template.xlsx
+++ b/corpus/templates/grouped-footers/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\foxtr\LocalTools\excel-graft\corpus\templates\grouped-footers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4191BB7-E249-4EE4-B911-DE9504B79FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{124E4D49-280D-4CBD-8803-398AC013E918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2240" yWindow="2470" windowWidth="28800" windowHeight="15910" xr2:uid="{947484D0-8180-4DF4-B8C1-15EE7FBBA707}"/>
+    <workbookView xWindow="2240" yWindow="2470" windowWidth="28800" windowHeight="15910" xr2:uid="{52CF7D76-8172-4C11-B328-8D6C04129C81}"/>
   </bookViews>
   <sheets>
     <sheet name="Payroll" sheetId="1" r:id="rId1"/>
@@ -528,7 +528,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56C03705-BE0F-42BF-96B6-64A2F5334D76}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9D737A6-230A-4059-AD3C-27CB14DEAA86}">
   <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>